<commit_message>
feat: expand data foundation to 22,584 records with 135+ canonical variables and multi-source calibration
</commit_message>
<xml_diff>
--- a/reports/policy_data_compatibility_report.xlsx
+++ b/reports/policy_data_compatibility_report.xlsx
@@ -321,7 +321,7 @@
         </is>
       </c>
       <c r="G6">
-        <v>98.7083</v>
+        <v>98.6982</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="G9">
-        <v>98.7083</v>
+        <v>98.6982</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -549,11 +549,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>EXACT_AVAILABLE</t>
         </is>
       </c>
       <c r="E11">
-        <v>0.0</v>
+        <v>0.85</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="G11">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -605,11 +605,11 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SRC_NFHS5_IIPS_2019_21</t>
+          <t>SRC_NFHS5_TN_HEALTH</t>
         </is>
       </c>
       <c r="G12">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="G15">
-        <v>98.7083</v>
+        <v>98.6982</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -909,21 +909,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TN_YOUTH_EMPLOYMENT_ASSISTANCE</t>
+          <t>TN_EDUCATION_SKILLING</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SOCIAL_WELFARE</t>
+          <t>DEMOGRAPHICS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PARTIALLY_SUPPORTED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="D6">
-        <v>61.0</v>
+        <v>77.5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DEMOGRAPHICS</t>
+          <t>EDUCATION</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -952,57 +952,57 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>['age', 'district', 'state']</t>
+          <t>['age', 'district', 'education_level']</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TN_EDUCATION_SKILLING</t>
+          <t>TN_HEALTH_INSURANCE_TOPUP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EDUCATION</t>
+          <t>INCOME</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SUPPORTED</t>
+          <t>PARTIALLY_SUPPORTED</t>
         </is>
       </c>
       <c r="D8">
-        <v>77.5</v>
+        <v>55.0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>['age', 'district', 'education_level']</t>
+          <t>['district', 'household_income']</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TN_EDUCATION_SKILLING</t>
+          <t>TN_HEALTH_INSURANCE_TOPUP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SOCIAL_WELFARE</t>
+          <t>DEMOGRAPHICS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SUPPORTED</t>
+          <t>PARTIALLY_SUPPORTED</t>
         </is>
       </c>
       <c r="D9">
-        <v>67.5</v>
+        <v>55.0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>['age', 'district', 'state']</t>
+          <t>['district', 'state']</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>INCOME</t>
+          <t>HEALTH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1027,87 +1027,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>['district', 'household_income']</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TN_HEALTH_INSURANCE_TOPUP</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>DEMOGRAPHICS</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>PARTIALLY_SUPPORTED</t>
-        </is>
-      </c>
-      <c r="D11">
-        <v>55.0</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>['district', 'state']</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TN_HEALTH_INSURANCE_TOPUP</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SOCIAL_WELFARE</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>PARTIALLY_SUPPORTED</t>
-        </is>
-      </c>
-      <c r="D12">
-        <v>55.0</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>['district', 'state']</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>TN_HEALTH_INSURANCE_TOPUP</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HEALTH</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>SUPPORTED</t>
-        </is>
-      </c>
-      <c r="D13">
-        <v>69.0</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>['disability_status', 'district', 'health_insurance']</t>
+          <t>['district', 'health_insurance']</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E10"/>
 </worksheet>
 </file>
 
@@ -1173,7 +1098,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>60.2</v>
+        <v>60.0</v>
       </c>
       <c r="C2">
         <v>73.34</v>
@@ -1194,7 +1119,7 @@
         <v>85.0</v>
       </c>
       <c r="I2">
-        <v>82.66</v>
+        <v>82.63</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1209,13 +1134,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>74.17</v>
+        <v>77.5</v>
       </c>
       <c r="C3">
         <v>84.5</v>
       </c>
       <c r="D3">
-        <v>99.68</v>
+        <v>99.67</v>
       </c>
       <c r="E3">
         <v>100.0</v>
@@ -1230,7 +1155,7 @@
         <v>85.0</v>
       </c>
       <c r="I3">
-        <v>89.69</v>
+        <v>90.18</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1245,13 +1170,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>58.5</v>
+        <v>55.0</v>
       </c>
       <c r="C4">
-        <v>42.07</v>
+        <v>59.07</v>
       </c>
       <c r="D4">
-        <v>48.74</v>
+        <v>74.74</v>
       </c>
       <c r="E4">
         <v>75.0</v>
@@ -1266,7 +1191,7 @@
         <v>88.0</v>
       </c>
       <c r="I4">
-        <v>62.59</v>
+        <v>71.51</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1478,7 +1403,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Acquire row-level health_insurance data before simulation.</t>
+          <t>Acquire row-level disability_status data before simulation.</t>
         </is>
       </c>
     </row>
@@ -1490,23 +1415,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Acquire row-level disability_status data before simulation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TN_HEALTH_INSURANCE_TOPUP</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
           <t>Treat household_income as a proxy-backed limitation; collect direct source data if eligibility depends on it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B6"/>
 </worksheet>
 </file>
</xml_diff>